<commit_message>
[fix/HD-15322] fix: Add the relevant report with site, zone and deployment name
</commit_message>
<xml_diff>
--- a/api/templates/critical_errors_by_module/en.xlsx
+++ b/api/templates/critical_errors_by_module/en.xlsx
@@ -10,14 +10,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="VMryN2BO/nCJB83XL3J+MRSFoUDeSphB++5JYslFESQ="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="I1Oz24h/bbGmTuXdU63Jux5pNwGb4wiGElkUZGzLihQ="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="65">
   <si>
     <t>Errors by Module</t>
   </si>
@@ -34,6 +34,12 @@
     <t>&lt;SitesLabel&gt;: &lt;Sites&gt;</t>
   </si>
   <si>
+    <t>&lt;Table&gt;</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
     <t>Deployment Name</t>
   </si>
   <si>
@@ -70,6 +76,9 @@
     <t>Total Errors During Period</t>
   </si>
   <si>
+    <t>&lt;#&gt;</t>
+  </si>
+  <si>
     <t>&lt;deploymentName&gt;</t>
   </si>
   <si>
@@ -100,10 +109,10 @@
     <t>&lt;errorDescription&gt;</t>
   </si>
   <si>
-    <t>&lt;totalRestsRunDuringPeriod&gt;</t>
-  </si>
-  <si>
-    <t>&lt;totalErrorsDuringPeriod&gt;</t>
+    <t>&lt;totalTests&gt;</t>
+  </si>
+  <si>
+    <t>&lt;totalErrors&gt;</t>
   </si>
   <si>
     <t>Code</t>
@@ -209,7 +218,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="12.0"/>
       <color rgb="FF000000"/>
@@ -232,6 +241,11 @@
       <sz val="12.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -260,8 +274,33 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
     <border>
       <left style="medium">
         <color rgb="FF000000"/>
@@ -280,7 +319,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -299,28 +338,35 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="2" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="3" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="3" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="3" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -543,8 +589,8 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="22.78"/>
-    <col customWidth="1" min="2" max="2" width="10.33"/>
+    <col customWidth="1" min="1" max="1" width="18.0"/>
+    <col customWidth="1" min="2" max="2" width="28.56"/>
     <col customWidth="1" min="3" max="3" width="10.67"/>
     <col customWidth="1" min="4" max="4" width="16.22"/>
     <col customWidth="1" min="5" max="5" width="14.22"/>
@@ -555,6 +601,7 @@
     <col customWidth="1" min="10" max="10" width="20.33"/>
     <col customWidth="1" min="11" max="11" width="28.44"/>
     <col customWidth="1" min="12" max="12" width="24.56"/>
+    <col customWidth="1" min="13" max="13" width="21.56"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -627,90 +674,102 @@
       <c r="G6" s="4"/>
       <c r="H6" s="5"/>
     </row>
-    <row r="7" ht="33.0" customHeight="1">
+    <row r="7">
       <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="5"/>
+    </row>
+    <row r="8" ht="33.0" customHeight="1">
+      <c r="A8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="B8" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="C8" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="D8" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="E8" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="F8" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="G8" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="H8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="J7" s="10" t="s">
+      <c r="I8" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="10" t="s">
+      <c r="J8" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="L7" s="10" t="s">
+      <c r="K8" s="13" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="s">
+      <c r="L8" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="M8" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="11" t="s">
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="B9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="C9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="D9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="E9" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="F9" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="G9" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="J8" s="12" t="s">
+      <c r="H9" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="K8" s="12" t="s">
+      <c r="I9" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="L8" s="12" t="s">
+      <c r="J9" s="14" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="5"/>
+      <c r="K9" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="M9" s="14" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="10">
+      <c r="B10" s="15"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
@@ -780,7 +839,7 @@
       <c r="G19" s="4"/>
       <c r="H19" s="5"/>
     </row>
-    <row r="20" ht="15.75" customHeight="1">
+    <row r="20">
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
@@ -2180,7 +2239,13 @@
       <c r="G219" s="4"/>
       <c r="H219" s="5"/>
     </row>
-    <row r="220" ht="15.75" customHeight="1"/>
+    <row r="220" ht="15.75" customHeight="1">
+      <c r="D220" s="4"/>
+      <c r="E220" s="4"/>
+      <c r="F220" s="4"/>
+      <c r="G220" s="4"/>
+      <c r="H220" s="5"/>
+    </row>
     <row r="221" ht="15.75" customHeight="1"/>
     <row r="222" ht="15.75" customHeight="1"/>
     <row r="223" ht="15.75" customHeight="1"/>
@@ -2960,6 +3025,7 @@
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -2982,300 +3048,300 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>31</v>
+      <c r="A1" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14">
+      <c r="A2" s="17">
         <v>1001.0</v>
       </c>
-      <c r="B2" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>33</v>
+      <c r="B2" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14">
+      <c r="A3" s="17">
         <v>1002.0</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>34</v>
+      <c r="B3" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14">
+      <c r="A4" s="17">
         <v>1004.0</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="14" t="s">
+      <c r="B4" s="17" t="s">
         <v>35</v>
       </c>
+      <c r="C4" s="17" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="14">
+      <c r="A5" s="17">
         <v>1005.0</v>
       </c>
-      <c r="B5" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>36</v>
+      <c r="B5" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14">
+      <c r="A6" s="17">
         <v>1006.0</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>37</v>
+      <c r="B6" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14">
+      <c r="A7" s="17">
         <v>1007.0</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>38</v>
+      <c r="B7" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14">
+      <c r="A8" s="17">
         <v>1017.0</v>
       </c>
-      <c r="B8" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>39</v>
+      <c r="B8" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14">
+      <c r="A9" s="17">
         <v>1018.0</v>
       </c>
-      <c r="B9" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>40</v>
+      <c r="B9" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14">
+      <c r="A10" s="17">
         <v>2003.0</v>
       </c>
-      <c r="B10" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>42</v>
+      <c r="B10" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14">
+      <c r="A11" s="17">
         <v>2005.0</v>
       </c>
-      <c r="B11" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>43</v>
+      <c r="B11" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14">
+      <c r="A12" s="17">
         <v>2008.0</v>
       </c>
-      <c r="B12" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C12" s="14" t="s">
+      <c r="B12" s="17" t="s">
         <v>44</v>
       </c>
+      <c r="C12" s="17" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="14">
+      <c r="A13" s="17">
         <v>2009.0</v>
       </c>
-      <c r="B13" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>45</v>
+      <c r="B13" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14">
+      <c r="A14" s="17">
         <v>2011.0</v>
       </c>
-      <c r="B14" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>47</v>
+      <c r="B14" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14">
+      <c r="A15" s="17">
         <v>2014.0</v>
       </c>
-      <c r="B15" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C15" s="14" t="s">
-        <v>48</v>
+      <c r="B15" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14">
+      <c r="A16" s="17">
         <v>2016.0</v>
       </c>
-      <c r="B16" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C16" s="14" t="s">
+      <c r="B16" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17">
+        <v>2018.0</v>
+      </c>
+      <c r="B17" s="17" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="14">
-        <v>2018.0</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>50</v>
+      <c r="C17" s="17" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14">
+      <c r="A18" s="17">
         <v>2022.0</v>
       </c>
-      <c r="B18" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C18" s="14" t="s">
+      <c r="B18" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17">
+        <v>2025.0</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17">
+        <v>2032.0</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="17">
+        <v>2034.0</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="17">
+        <v>2037.0</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="17">
+        <v>4010.0</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="17">
+        <v>4017.0</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" s="17" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="14">
-        <v>2025.0</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="14">
-        <v>2032.0</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="14">
-        <v>2034.0</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="14">
-        <v>2037.0</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="14">
-        <v>4010.0</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="14">
-        <v>4017.0</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>48</v>
-      </c>
-    </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="14">
+      <c r="A25" s="17">
         <v>5006.0</v>
       </c>
-      <c r="B25" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>59</v>
+      <c r="B25" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="14">
+      <c r="A26" s="17">
         <v>5007.0</v>
       </c>
-      <c r="B26" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>60</v>
+      <c r="B26" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="14">
+      <c r="A27" s="17">
         <v>5011.0</v>
       </c>
-      <c r="B27" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C27" s="14" t="s">
+      <c r="B27" s="17" t="s">
         <v>61</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
[feat/HD-15370] refactor: update the report and remove error category in it
</commit_message>
<xml_diff>
--- a/api/templates/critical_errors_by_module/en.xlsx
+++ b/api/templates/critical_errors_by_module/en.xlsx
@@ -10,14 +10,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="I1Oz24h/bbGmTuXdU63Jux5pNwGb4wiGElkUZGzLihQ="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="F6mb/vCgUweCCWf2LUZubW8whLIJiDMIUq8lQcBJcxA="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="63">
   <si>
     <t>Errors by Module</t>
   </si>
@@ -64,9 +64,6 @@
     <t>Error code</t>
   </si>
   <si>
-    <t>Error Category</t>
-  </si>
-  <si>
     <t>Error description</t>
   </si>
   <si>
@@ -101,9 +98,6 @@
   </si>
   <si>
     <t>&lt;errorCode&gt;</t>
-  </si>
-  <si>
-    <t>&lt;errorCategory&gt;</t>
   </si>
   <si>
     <t>&lt;errorDescription&gt;</t>
@@ -319,7 +313,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -357,9 +351,6 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -598,10 +589,9 @@
     <col customWidth="1" min="7" max="7" width="11.78"/>
     <col customWidth="1" min="8" max="8" width="11.67"/>
     <col customWidth="1" min="9" max="9" width="17.67"/>
-    <col customWidth="1" min="10" max="10" width="20.33"/>
-    <col customWidth="1" min="11" max="11" width="28.44"/>
-    <col customWidth="1" min="12" max="12" width="24.56"/>
-    <col customWidth="1" min="13" max="13" width="21.56"/>
+    <col customWidth="1" min="10" max="10" width="28.44"/>
+    <col customWidth="1" min="11" max="11" width="24.56"/>
+    <col customWidth="1" min="12" max="12" width="21.56"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -717,59 +707,53 @@
       <c r="J8" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="K8" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="L8" s="13" t="s">
+      <c r="L8" s="12" t="s">
         <v>17</v>
-      </c>
-      <c r="M8" s="13" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="F9" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="G9" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="H9" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="I9" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="I9" s="14" t="s">
+      <c r="J9" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="J9" s="14" t="s">
+      <c r="K9" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="K9" s="14" t="s">
+      <c r="L9" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="L9" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="M9" s="14" t="s">
-        <v>31</v>
-      </c>
     </row>
     <row r="10">
-      <c r="B10" s="15"/>
+      <c r="B10" s="14"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
@@ -3048,300 +3032,300 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="16" t="s">
+    </row>
+    <row r="2">
+      <c r="A2" s="16">
+        <v>1001.0</v>
+      </c>
+      <c r="B2" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C2" s="16" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="17">
-        <v>1001.0</v>
-      </c>
-      <c r="B2" s="17" t="s">
+    <row r="3">
+      <c r="A3" s="16">
+        <v>1002.0</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="17" t="s">
+    </row>
+    <row r="4">
+      <c r="A4" s="16">
+        <v>1004.0</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="16" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="17">
-        <v>1002.0</v>
-      </c>
-      <c r="B3" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" s="17" t="s">
+    <row r="5">
+      <c r="A5" s="16">
+        <v>1005.0</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="16" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="17">
-        <v>1004.0</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="17" t="s">
+    <row r="6">
+      <c r="A6" s="16">
+        <v>1006.0</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="16" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="17">
-        <v>1005.0</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="17" t="s">
+    <row r="7">
+      <c r="A7" s="16">
+        <v>1007.0</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="16" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="17">
-        <v>1006.0</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="17" t="s">
+    <row r="8">
+      <c r="A8" s="16">
+        <v>1017.0</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="16" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="17">
-        <v>1007.0</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="17" t="s">
+    <row r="9">
+      <c r="A9" s="16">
+        <v>1018.0</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="16" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="17">
-        <v>1017.0</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="17" t="s">
+    <row r="10">
+      <c r="A10" s="16">
+        <v>2003.0</v>
+      </c>
+      <c r="B10" s="16" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="17">
-        <v>1018.0</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="17" t="s">
+      <c r="C10" s="16" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="17">
-        <v>2003.0</v>
-      </c>
-      <c r="B10" s="17" t="s">
+    <row r="11">
+      <c r="A11" s="16">
+        <v>2005.0</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="17" t="s">
+    </row>
+    <row r="12">
+      <c r="A12" s="16">
+        <v>2008.0</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="16" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="17">
-        <v>2005.0</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="17" t="s">
+    <row r="13">
+      <c r="A13" s="16">
+        <v>2009.0</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="16" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="17">
-        <v>2008.0</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="17" t="s">
+    <row r="14">
+      <c r="A14" s="16">
+        <v>2011.0</v>
+      </c>
+      <c r="B14" s="16" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="17">
-        <v>2009.0</v>
-      </c>
-      <c r="B13" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" s="17" t="s">
+      <c r="C14" s="16" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="17">
-        <v>2011.0</v>
-      </c>
-      <c r="B14" s="17" t="s">
+    <row r="15">
+      <c r="A15" s="16">
+        <v>2014.0</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="17" t="s">
+    </row>
+    <row r="16">
+      <c r="A16" s="16">
+        <v>2016.0</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="16" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="17">
-        <v>2014.0</v>
-      </c>
-      <c r="B15" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="17" t="s">
+    <row r="17">
+      <c r="A17" s="16">
+        <v>2018.0</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="16" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="17">
-        <v>2016.0</v>
-      </c>
-      <c r="B16" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C16" s="17" t="s">
+    <row r="18">
+      <c r="A18" s="16">
+        <v>2022.0</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" s="16" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="17">
-        <v>2018.0</v>
-      </c>
-      <c r="B17" s="17" t="s">
+    <row r="19">
+      <c r="A19" s="16">
+        <v>2025.0</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16">
+        <v>2032.0</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="16">
+        <v>2034.0</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="16">
+        <v>2037.0</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="16">
+        <v>4010.0</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="16">
+        <v>4017.0</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="17">
-        <v>2022.0</v>
-      </c>
-      <c r="B18" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="17" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="17">
-        <v>2025.0</v>
-      </c>
-      <c r="B19" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C19" s="17" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="17">
-        <v>2032.0</v>
-      </c>
-      <c r="B20" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C20" s="17" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="17">
-        <v>2034.0</v>
-      </c>
-      <c r="B21" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C21" s="17" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="17">
-        <v>2037.0</v>
-      </c>
-      <c r="B22" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C22" s="17" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="17">
-        <v>4010.0</v>
-      </c>
-      <c r="B23" s="17" t="s">
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="16">
+        <v>5006.0</v>
+      </c>
+      <c r="B25" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C25" s="16" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="17">
-        <v>4017.0</v>
-      </c>
-      <c r="B24" s="17" t="s">
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="16">
+        <v>5007.0</v>
+      </c>
+      <c r="B26" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="17" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="17">
-        <v>5006.0</v>
-      </c>
-      <c r="B25" s="17" t="s">
+      <c r="C26" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="C25" s="17" t="s">
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="16">
+        <v>5011.0</v>
+      </c>
+      <c r="B27" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" s="16" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="17">
-        <v>5007.0</v>
-      </c>
-      <c r="B26" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="C26" s="17" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="17">
-        <v>5011.0</v>
-      </c>
-      <c r="B27" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="C27" s="17" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
[feat/HD-15370] fix: remove the error description from the sheet
</commit_message>
<xml_diff>
--- a/api/templates/critical_errors_by_module/en.xlsx
+++ b/api/templates/critical_errors_by_module/en.xlsx
@@ -10,14 +10,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="F6mb/vCgUweCCWf2LUZubW8whLIJiDMIUq8lQcBJcxA="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="SJ8YGPqmPeu7bFouTkualnmYW15Z2N2hd9k8S3BpbXs="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="61">
   <si>
     <t>Errors by Module</t>
   </si>
@@ -64,9 +64,6 @@
     <t>Error code</t>
   </si>
   <si>
-    <t>Error description</t>
-  </si>
-  <si>
     <t>Total Tests Run During Period</t>
   </si>
   <si>
@@ -98,9 +95,6 @@
   </si>
   <si>
     <t>&lt;errorCode&gt;</t>
-  </si>
-  <si>
-    <t>&lt;errorDescription&gt;</t>
   </si>
   <si>
     <t>&lt;totalTests&gt;</t>
@@ -589,9 +583,8 @@
     <col customWidth="1" min="7" max="7" width="11.78"/>
     <col customWidth="1" min="8" max="8" width="11.67"/>
     <col customWidth="1" min="9" max="9" width="17.67"/>
-    <col customWidth="1" min="10" max="10" width="28.44"/>
-    <col customWidth="1" min="11" max="11" width="24.56"/>
-    <col customWidth="1" min="12" max="12" width="21.56"/>
+    <col customWidth="1" min="10" max="10" width="24.56"/>
+    <col customWidth="1" min="11" max="11" width="21.56"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -710,46 +703,40 @@
       <c r="K8" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="L8" s="12" t="s">
-        <v>17</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="F9" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="G9" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="H9" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="I9" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="J9" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="K9" s="13" t="s">
         <v>27</v>
-      </c>
-      <c r="K9" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="L9" s="13" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="10">
@@ -3033,13 +3020,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="15" t="s">
         <v>30</v>
-      </c>
-      <c r="B1" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="15" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="2">
@@ -3047,10 +3034,10 @@
         <v>1001.0</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -3058,10 +3045,10 @@
         <v>1002.0</v>
       </c>
       <c r="B3" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="16" t="s">
         <v>33</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="4">
@@ -3069,10 +3056,10 @@
         <v>1004.0</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
@@ -3080,10 +3067,10 @@
         <v>1005.0</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -3091,10 +3078,10 @@
         <v>1006.0</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
@@ -3102,10 +3089,10 @@
         <v>1007.0</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8">
@@ -3113,10 +3100,10 @@
         <v>1017.0</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9">
@@ -3124,10 +3111,10 @@
         <v>1018.0</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10">
@@ -3135,10 +3122,10 @@
         <v>2003.0</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11">
@@ -3146,10 +3133,10 @@
         <v>2005.0</v>
       </c>
       <c r="B11" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="16" t="s">
         <v>42</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="12">
@@ -3157,10 +3144,10 @@
         <v>2008.0</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13">
@@ -3168,10 +3155,10 @@
         <v>2009.0</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14">
@@ -3179,10 +3166,10 @@
         <v>2011.0</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15">
@@ -3190,10 +3177,10 @@
         <v>2014.0</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16">
@@ -3201,10 +3188,10 @@
         <v>2016.0</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17">
@@ -3212,10 +3199,10 @@
         <v>2018.0</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18">
@@ -3223,10 +3210,10 @@
         <v>2022.0</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19">
@@ -3234,10 +3221,10 @@
         <v>2025.0</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="20">
@@ -3245,10 +3232,10 @@
         <v>2032.0</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -3256,10 +3243,10 @@
         <v>2034.0</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -3267,10 +3254,10 @@
         <v>2037.0</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -3278,10 +3265,10 @@
         <v>4010.0</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -3289,10 +3276,10 @@
         <v>4017.0</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
@@ -3300,10 +3287,10 @@
         <v>5006.0</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -3311,10 +3298,10 @@
         <v>5007.0</v>
       </c>
       <c r="B26" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" s="16" t="s">
         <v>59</v>
-      </c>
-      <c r="C26" s="16" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
@@ -3322,10 +3309,10 @@
         <v>5011.0</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>

</xml_diff>